<commit_message>
Regenerate core_profiles_history.xlsx for the #1979 confinement columns
#1979 added v_res_V, p_ohm_MW, p_net_MW, w_mhd_kJ and tau_e_net_s to the
core_profiles summary preset without regenerating the checked-in sheet, so
test_checked_in_sheet_matches_its_summary_preset[gen_core_profiles_history]
failed on both legs of the full Package CI (run 38170407038). Rebuilt as in
#1843 from the public source (the only one holding core_profiles) over
39900-40400: 12 rows, shots 39915/39916/40330, every preset column present.
The five new columns are empty for these shots -- their chain needs inputs
the public source does not carry -- which the gate does not mind (it checks
columns) and the sheet now states truthfully.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/workflow/automatic_pipeline_3_data_summary/core_profiles_history.xlsx
+++ b/workflow/automatic_pipeline_3_data_summary/core_profiles_history.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$T$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$Y$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T13"/>
+  <dimension ref="A1:Y13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -445,12 +445,17 @@
     <col width="14" customWidth="1" min="12" max="12"/>
     <col width="19" customWidth="1" min="13" max="13"/>
     <col width="22" customWidth="1" min="14" max="14"/>
-    <col width="17" customWidth="1" min="15" max="15"/>
-    <col width="19" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
     <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="16" customWidth="1" min="18" max="18"/>
-    <col width="22" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="16" customWidth="1" min="23" max="23"/>
+    <col width="22" customWidth="1" min="24" max="24"/>
+    <col width="12" customWidth="1" min="25" max="25"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -526,30 +531,55 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
+          <t>v_res_V</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>p_ohm_MW</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>p_net_MW</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>w_mhd_kJ</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>tau_e_net_s</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
           <t>ne_line_1e19_m3</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>ne_volume_1e19_m3</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>te_mean_eV</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>major_radius_m</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>inverse_aspect_ratio</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="Y1" s="1" t="inlineStr">
         <is>
           <t>elongation</t>
         </is>
@@ -595,22 +625,27 @@
       <c r="N2" s="3" t="n">
         <v>0.0006056141613133538</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="O2" s="3" t="n"/>
+      <c r="P2" s="3" t="n"/>
+      <c r="Q2" s="3" t="n"/>
+      <c r="R2" s="3" t="n"/>
+      <c r="S2" s="3" t="n"/>
+      <c r="T2" s="3" t="n">
         <v>0.397137554447844</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="U2" s="3" t="n">
         <v>0.2770392005620234</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="V2" s="3" t="n">
         <v>109.3738925206001</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="W2" s="3" t="n">
         <v>0.39945373685</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="X2" s="3" t="n">
         <v>0.7339450044000759</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="Y2" s="3" t="n">
         <v>1.534159114388222</v>
       </c>
     </row>
@@ -654,22 +689,27 @@
       <c r="N3" s="3" t="n">
         <v>0.0005568729755057317</v>
       </c>
-      <c r="O3" s="3" t="n">
+      <c r="O3" s="3" t="n"/>
+      <c r="P3" s="3" t="n"/>
+      <c r="Q3" s="3" t="n"/>
+      <c r="R3" s="3" t="n"/>
+      <c r="S3" s="3" t="n"/>
+      <c r="T3" s="3" t="n">
         <v>0.511561602940355</v>
       </c>
-      <c r="P3" s="3" t="n">
+      <c r="U3" s="3" t="n">
         <v>0.3123892042000352</v>
       </c>
-      <c r="Q3" s="3" t="n">
+      <c r="V3" s="3" t="n">
         <v>94.87967221362184</v>
       </c>
-      <c r="R3" s="3" t="n">
+      <c r="W3" s="3" t="n">
         <v>0.37307581435</v>
       </c>
-      <c r="S3" s="3" t="n">
+      <c r="X3" s="3" t="n">
         <v>0.7158513438221756</v>
       </c>
-      <c r="T3" s="3" t="n">
+      <c r="Y3" s="3" t="n">
         <v>1.536035386291677</v>
       </c>
     </row>
@@ -713,22 +753,27 @@
       <c r="N4" s="3" t="n">
         <v>0.0008530621968854026</v>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="O4" s="3" t="n"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
+      <c r="S4" s="3" t="n"/>
+      <c r="T4" s="3" t="n">
         <v>0.3614876345372368</v>
       </c>
-      <c r="P4" s="3" t="n">
+      <c r="U4" s="3" t="n">
         <v>0.2482699587978707</v>
       </c>
-      <c r="Q4" s="3" t="n">
+      <c r="V4" s="3" t="n">
         <v>112.7496930888605</v>
       </c>
-      <c r="R4" s="3" t="n">
+      <c r="W4" s="3" t="n">
         <v>0.39460676245</v>
       </c>
-      <c r="S4" s="3" t="n">
+      <c r="X4" s="3" t="n">
         <v>0.7307929156093458</v>
       </c>
-      <c r="T4" s="3" t="n">
+      <c r="Y4" s="3" t="n">
         <v>1.525839609236771</v>
       </c>
     </row>
@@ -772,22 +817,27 @@
       <c r="N5" s="3" t="n">
         <v>0.0007380317652458885</v>
       </c>
-      <c r="O5" s="3" t="n">
+      <c r="O5" s="3" t="n"/>
+      <c r="P5" s="3" t="n"/>
+      <c r="Q5" s="3" t="n"/>
+      <c r="R5" s="3" t="n"/>
+      <c r="S5" s="3" t="n"/>
+      <c r="T5" s="3" t="n">
         <v>0.5131336735365954</v>
       </c>
-      <c r="P5" s="3" t="n">
+      <c r="U5" s="3" t="n">
         <v>0.3298516714144583</v>
       </c>
-      <c r="Q5" s="3" t="n">
+      <c r="V5" s="3" t="n">
         <v>109.8348040456633</v>
       </c>
-      <c r="R5" s="3" t="n">
+      <c r="W5" s="3" t="n">
         <v>0.37916388135</v>
       </c>
-      <c r="S5" s="3" t="n">
+      <c r="X5" s="3" t="n">
         <v>0.7202496961938011</v>
       </c>
-      <c r="T5" s="3" t="n">
+      <c r="Y5" s="3" t="n">
         <v>1.535903916808337</v>
       </c>
     </row>
@@ -831,22 +881,27 @@
       <c r="N6" s="3" t="n">
         <v>0.0004547147690028754</v>
       </c>
-      <c r="O6" s="3" t="n">
+      <c r="O6" s="3" t="n"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
+      <c r="S6" s="3" t="n"/>
+      <c r="T6" s="3" t="n">
         <v>0.4252888665215075</v>
       </c>
-      <c r="P6" s="3" t="n">
+      <c r="U6" s="3" t="n">
         <v>0.3175637437653519</v>
       </c>
-      <c r="Q6" s="3" t="n">
+      <c r="V6" s="3" t="n">
         <v>102.0212249530595</v>
       </c>
-      <c r="R6" s="3" t="n">
+      <c r="W6" s="3" t="n">
         <v>0.3663759888</v>
       </c>
-      <c r="S6" s="3" t="n">
+      <c r="X6" s="3" t="n">
         <v>0.7108559167674364</v>
       </c>
-      <c r="T6" s="3" t="n">
+      <c r="Y6" s="3" t="n">
         <v>1.530831081418437</v>
       </c>
     </row>
@@ -890,22 +945,27 @@
       <c r="N7" s="3" t="n">
         <v>0.0004969304101282553</v>
       </c>
-      <c r="O7" s="3" t="n">
+      <c r="O7" s="3" t="n"/>
+      <c r="P7" s="3" t="n"/>
+      <c r="Q7" s="3" t="n"/>
+      <c r="R7" s="3" t="n"/>
+      <c r="S7" s="3" t="n"/>
+      <c r="T7" s="3" t="n">
         <v>0.3894290255701583</v>
       </c>
-      <c r="P7" s="3" t="n">
+      <c r="U7" s="3" t="n">
         <v>0.2279634101701252</v>
       </c>
-      <c r="Q7" s="3" t="n">
+      <c r="V7" s="3" t="n">
         <v>95.85426222679759</v>
       </c>
-      <c r="R7" s="3" t="n">
+      <c r="W7" s="3" t="n">
         <v>0.35110020495</v>
       </c>
-      <c r="S7" s="3" t="n">
+      <c r="X7" s="3" t="n">
         <v>0.6987051029632274</v>
       </c>
-      <c r="T7" s="3" t="n">
+      <c r="Y7" s="3" t="n">
         <v>1.523715455812232</v>
       </c>
     </row>
@@ -949,22 +1009,27 @@
       <c r="N8" s="3" t="n">
         <v>0.00335602447917664</v>
       </c>
-      <c r="O8" s="3" t="n">
+      <c r="O8" s="3" t="n"/>
+      <c r="P8" s="3" t="n"/>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="3" t="n"/>
+      <c r="S8" s="3" t="n"/>
+      <c r="T8" s="3" t="n">
         <v>0.4790600170522634</v>
       </c>
-      <c r="P8" s="3" t="n">
+      <c r="U8" s="3" t="n">
         <v>0.3232492246319317</v>
       </c>
-      <c r="Q8" s="3" t="n">
+      <c r="V8" s="3" t="n">
         <v>155.3721236549243</v>
       </c>
-      <c r="R8" s="3" t="n">
+      <c r="W8" s="3" t="n">
         <v>0.3380066516</v>
       </c>
-      <c r="S8" s="3" t="n">
+      <c r="X8" s="3" t="n">
         <v>0.6873735691300815</v>
       </c>
-      <c r="T8" s="3" t="n">
+      <c r="Y8" s="3" t="n">
         <v>1.51286038491215</v>
       </c>
     </row>
@@ -1008,22 +1073,27 @@
       <c r="N9" s="3" t="n">
         <v>0.0004108297961651184</v>
       </c>
-      <c r="O9" s="3" t="n">
+      <c r="O9" s="3" t="n"/>
+      <c r="P9" s="3" t="n"/>
+      <c r="Q9" s="3" t="n"/>
+      <c r="R9" s="3" t="n"/>
+      <c r="S9" s="3" t="n"/>
+      <c r="T9" s="3" t="n">
         <v>0.5861270972150804</v>
       </c>
-      <c r="P9" s="3" t="n">
+      <c r="U9" s="3" t="n">
         <v>0.5970951570111389</v>
       </c>
-      <c r="Q9" s="3" t="n">
+      <c r="V9" s="3" t="n">
         <v>112.9036858442067</v>
       </c>
-      <c r="R9" s="3" t="n">
+      <c r="W9" s="3" t="n">
         <v>0.30854622985</v>
       </c>
-      <c r="S9" s="3" t="n">
+      <c r="X9" s="3" t="n">
         <v>0.6583209256802396</v>
       </c>
-      <c r="T9" s="3" t="n">
+      <c r="Y9" s="3" t="n">
         <v>1.481995351687039</v>
       </c>
     </row>
@@ -1067,22 +1137,27 @@
       <c r="N10" s="3" t="n">
         <v>0.0005603904324370252</v>
       </c>
-      <c r="O10" s="3" t="n">
+      <c r="O10" s="3" t="n"/>
+      <c r="P10" s="3" t="n"/>
+      <c r="Q10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
+      <c r="S10" s="3" t="n"/>
+      <c r="T10" s="3" t="n">
         <v>0.6113545034881003</v>
       </c>
-      <c r="P10" s="3" t="n">
+      <c r="U10" s="3" t="n">
         <v>0.6074394177922189</v>
       </c>
-      <c r="Q10" s="3" t="n">
+      <c r="V10" s="3" t="n">
         <v>254.3577280189549</v>
       </c>
-      <c r="R10" s="3" t="n">
+      <c r="W10" s="3" t="n">
         <v>0.2583589832</v>
       </c>
-      <c r="S10" s="3" t="n">
+      <c r="X10" s="3" t="n">
         <v>0.5934888913125278</v>
       </c>
-      <c r="T10" s="3" t="n">
+      <c r="Y10" s="3" t="n">
         <v>1.401551608634724</v>
       </c>
     </row>
@@ -1126,22 +1201,27 @@
       <c r="N11" s="3" t="n">
         <v>0.0005047169387639488</v>
       </c>
-      <c r="O11" s="3" t="n">
+      <c r="O11" s="3" t="n"/>
+      <c r="P11" s="3" t="n"/>
+      <c r="Q11" s="3" t="n"/>
+      <c r="R11" s="3" t="n"/>
+      <c r="S11" s="3" t="n"/>
+      <c r="T11" s="3" t="n">
         <v>1.546542601406171</v>
       </c>
-      <c r="P11" s="3" t="n">
+      <c r="U11" s="3" t="n">
         <v>1.272407731542776</v>
       </c>
-      <c r="Q11" s="3" t="n">
+      <c r="V11" s="3" t="n">
         <v>33.65089447856616</v>
       </c>
-      <c r="R11" s="3" t="n">
+      <c r="W11" s="3" t="n">
         <v>0.3691923345</v>
       </c>
-      <c r="S11" s="3" t="n">
+      <c r="X11" s="3" t="n">
         <v>0.7130232204211705</v>
       </c>
-      <c r="T11" s="3" t="n">
+      <c r="Y11" s="3" t="n">
         <v>1.492828742026219</v>
       </c>
     </row>
@@ -1185,22 +1265,27 @@
       <c r="N12" s="3" t="n">
         <v>0.0003648862449745406</v>
       </c>
-      <c r="O12" s="3" t="n">
+      <c r="O12" s="3" t="n"/>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="n"/>
+      <c r="R12" s="3" t="n"/>
+      <c r="S12" s="3" t="n"/>
+      <c r="T12" s="3" t="n">
         <v>1.768135037031632</v>
       </c>
-      <c r="P12" s="3" t="n">
+      <c r="U12" s="3" t="n">
         <v>1.428777154123582</v>
       </c>
-      <c r="Q12" s="3" t="n">
+      <c r="V12" s="3" t="n">
         <v>34.99929264514812</v>
       </c>
-      <c r="R12" s="3" t="n">
+      <c r="W12" s="3" t="n">
         <v>0.31948140835</v>
       </c>
-      <c r="S12" s="3" t="n">
+      <c r="X12" s="3" t="n">
         <v>0.6697696750340497</v>
       </c>
-      <c r="T12" s="3" t="n">
+      <c r="Y12" s="3" t="n">
         <v>1.469919200986114</v>
       </c>
     </row>
@@ -1244,27 +1329,32 @@
       <c r="N13" s="3" t="n">
         <v>0.0003282194839591677</v>
       </c>
-      <c r="O13" s="3" t="n">
+      <c r="O13" s="3" t="n"/>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="3" t="n"/>
+      <c r="S13" s="3" t="n"/>
+      <c r="T13" s="3" t="n">
         <v>3.340954425158539</v>
       </c>
-      <c r="P13" s="3" t="n">
+      <c r="U13" s="3" t="n">
         <v>3.291312308711154</v>
       </c>
-      <c r="Q13" s="3" t="n">
+      <c r="V13" s="3" t="n">
         <v>46.84903230838708</v>
       </c>
-      <c r="R13" s="3" t="n">
+      <c r="W13" s="3" t="n">
         <v>0.2473906659</v>
       </c>
-      <c r="S13" s="3" t="n">
+      <c r="X13" s="3" t="n">
         <v>0.5758606254675189</v>
       </c>
-      <c r="T13" s="3" t="n">
+      <c r="Y13" s="3" t="n">
         <v>1.381928741049707</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T13"/>
+  <autoFilter ref="A1:Y13"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>